<commit_message>
Update PricingCalculator to include force_price_zero option in output generation when generation the output file for reverse; enhance main.py with default zone pricing creation and improved sheet processing logic.
</commit_message>
<xml_diff>
--- a/Courier_ids_Modes.xlsx
+++ b/Courier_ids_Modes.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prozo.PROZO-HO-1087\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prozo.PROZO-HO-1087\Downloads\Client onboarding automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -15,7 +15,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="52">
   <si>
     <t>Sheet Name</t>
   </si>
@@ -188,6 +188,12 @@
   </si>
   <si>
     <t>NDD</t>
+  </si>
+  <si>
+    <t>Reverse Air</t>
+  </si>
+  <si>
+    <t>Reverse Surface</t>
   </si>
 </sst>
 </file>
@@ -661,20 +667,20 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="14.5" thickBot="1">
+    <row r="10" spans="1:2" ht="28.5" thickBot="1">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="14.5" thickBot="1">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="28.5" thickBot="1">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="14.5" thickBot="1">
@@ -4766,6 +4772,7 @@
       <c r="B1000" s="1"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>